<commit_message>
Update delegation avg check to 87500 rub; add capacity note
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WQtgSHTUBUwP9xHzFTYxiY
</commit_message>
<xml_diff>
--- a/decomposition.xlsx
+++ b/decomposition.xlsx
@@ -746,7 +746,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -788,11 +788,11 @@
         </is>
       </c>
       <c r="B3" s="10" t="n">
-        <v>80000</v>
+        <v>87500</v>
       </c>
       <c r="C3" s="8" t="inlineStr">
         <is>
-          <t>← ПОД ВОПРОСОМ — уточнить</t>
+          <t>середина 75-100к</t>
         </is>
       </c>
     </row>
@@ -1035,8 +1035,16 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>• Срок 1 заказа делегирования: 2–3 недели → рост числа заказов = только через делегатов (параллельные потоки), не своим временем.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="7">
+    <mergeCell ref="A18:H18"/>
     <mergeCell ref="A15:H15"/>
     <mergeCell ref="A16:H16"/>
     <mergeCell ref="A13:H13"/>

</xml_diff>

<commit_message>
Finalize decomposition: filled expenses + income plan for 750k goal
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WQtgSHTUBUwP9xHzFTYxiY
</commit_message>
<xml_diff>
--- a/decomposition.xlsx
+++ b/decomposition.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="Расходы" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Доходы" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Сводка" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -105,7 +106,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -121,6 +122,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -728,7 +730,7 @@
     <row r="21">
       <c r="A21" s="8" t="inlineStr">
         <is>
-          <t>⚠ Жильё = 0: подтвердить, что нет аренды/ипотеки. Долги 22 200 = 266 400 ₽ ÷ 12 мес.</t>
+          <t>Допущение: жильё = 0 (нет аренды/ипотеки). Долги 22 200 = 266 400 ₽ ÷ 12 мес.</t>
         </is>
       </c>
     </row>
@@ -752,7 +754,7 @@
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="44" customWidth="1" min="2" max="2"/>
     <col width="9" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
@@ -775,11 +777,6 @@
       <c r="B2" s="10" t="n">
         <v>80</v>
       </c>
-      <c r="C2" s="8" t="inlineStr">
-        <is>
-          <t>← правь под актуальный</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
@@ -824,7 +821,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Цена/ед., ₽</t>
+          <t>Доход с ед., ₽</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -909,7 +906,7 @@
         <v/>
       </c>
       <c r="G8" s="4" t="n">
-        <v>408000</v>
+        <v>157500</v>
       </c>
       <c r="H8" s="12">
         <f>IF(D8=0,"—",ROUND(G8/D8,1))</f>
@@ -954,7 +951,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Академия / проекты RealMind (потенциал)</t>
+          <t>Академия / проекты RealMind</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
@@ -963,7 +960,7 @@
         </is>
       </c>
       <c r="D10" s="4" t="n">
-        <v>0</v>
+        <v>50000</v>
       </c>
       <c r="E10" s="3" t="n">
         <v>0</v>
@@ -973,7 +970,7 @@
         <v/>
       </c>
       <c r="G10" s="4" t="n">
-        <v>0</v>
+        <v>250500</v>
       </c>
       <c r="H10" s="12">
         <f>IF(D10=0,"—",ROUND(G10/D10,1))</f>
@@ -1003,42 +1000,42 @@
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>Пояснения:</t>
+          <t>Пояснения к плану (цель 750 000 ₽/мес):</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
         <is>
-          <t>• Гипнотерапия: $150/сессия × курс. Сейчас 4/мес, цель 16/мес (программа — цена может быть выше).</t>
+          <t>• Гипнотерапия: $150/сессия × курс 80. Рост 4 → 16 сессий/мес (программа, цена может быть выше).</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
         <is>
-          <t>• Делегирование: доход = 30% × средний чек. Сейчас ~3-4 заказа/мес (часть отменяется).</t>
+          <t>• Делегирование: 30% × 87 500 = 26 250 ₽/заказ. 1 заказ = 2–3 недели → рост числа заказов только через делегатов (параллельные потоки). В плане 6 заказов/мес по текущей мощности.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
         <is>
-          <t>• Почасовая: 2500 ₽/ч × ~10 ч/нед (≈43,3 ч/мес).</t>
+          <t>• Почасовая: 2 500 ₽/ч, рост до 60 ч/мес (~14 ч/нед).</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t>• «Нужно ед./мес» — сколько надо продать/отработать для плановой суммы.</t>
+          <t>• RealMind/Академия: цена проекта 50 000 ₽ — ЗАГЛУШКА, задать реальную. Этот канал закрывает разрыв цели (~250 500).</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t>• Срок 1 заказа делегирования: 2–3 недели → рост числа заказов = только через делегатов (параллельные потоки), не своим временем.</t>
+          <t>• «Нужно ед./мес» — сколько продать/отработать, чтобы выйти на плановую сумму.</t>
         </is>
       </c>
     </row>
@@ -1054,4 +1051,87 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>СВОДКА</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>Расходы, факт / мес</t>
+        </is>
+      </c>
+      <c r="B3" s="13">
+        <f>Расходы.C19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>Доход, факт / мес</t>
+        </is>
+      </c>
+      <c r="B4" s="13">
+        <f>Доходы.F11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>Профицит сейчас (доход − расход)</t>
+        </is>
+      </c>
+      <c r="B5" s="13">
+        <f>B4-B3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>Цель дохода / мес</t>
+        </is>
+      </c>
+      <c r="B6" s="13">
+        <f>Доходы.B4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>До цели (цель − факт дохода)</t>
+        </is>
+      </c>
+      <c r="B7" s="13">
+        <f>B6-B4</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:B1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>